<commit_message>
chore(backup): curadoria temática 2026-09-09
</commit_message>
<xml_diff>
--- a/backups/2026-09-09/marcacoes.xlsx
+++ b/backups/2026-09-09/marcacoes.xlsx
@@ -506,7 +506,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R2" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S2" t="str">
         <v>cmr9elunk0000a0igqhxlxb8n</v>
@@ -559,7 +559,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R3" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S3" t="str">
         <v>cmr9elunr0001a0igjnt49j4i</v>
@@ -612,7 +612,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R4" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S4" t="str">
         <v>cmr9elunr0002a0igmk8jsomc</v>
@@ -665,7 +665,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R5" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S5" t="str">
         <v>cmr9elunr0003a0ig4n49tro3</v>
@@ -718,7 +718,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R6" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S6" t="str">
         <v>cmr9elunr0004a0igegnj294a</v>
@@ -771,7 +771,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R7" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S7" t="str">
         <v>cmr9elunr0005a0igjykd6and</v>
@@ -824,7 +824,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R8" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S8" t="str">
         <v>cmr9elunr0006a0ig3lcgbjqt</v>
@@ -877,7 +877,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R9" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S9" t="str">
         <v>cmr9elunr0007a0ig0g6cpm20</v>
@@ -930,7 +930,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R10" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S10" t="str">
         <v>cmr9elunr0008a0ig5pe0z4qk</v>
@@ -983,7 +983,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R11" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S11" t="str">
         <v>cmr9eluns0009a0igzztvho7g</v>
@@ -1036,7 +1036,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R12" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S12" t="str">
         <v>cmr9eluns000aa0igpfobbt8c</v>
@@ -1089,7 +1089,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R13" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S13" t="str">
         <v>cmr9eluns000ba0ig61m6zcs2</v>
@@ -1142,7 +1142,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R14" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S14" t="str">
         <v>cmr9eluns000ca0igo78c7qf5</v>
@@ -1195,7 +1195,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R15" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S15" t="str">
         <v>cmr9eluns000da0ig6d8o9isj</v>
@@ -1248,7 +1248,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R16" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S16" t="str">
         <v>cmr9eluns000ea0igqm8pahyg</v>
@@ -1301,7 +1301,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R17" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S17" t="str">
         <v>cmr9eluns000fa0ig4ugvtzg2</v>
@@ -1354,7 +1354,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R18" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S18" t="str">
         <v>cmr9eluns000ga0igxraik2b0</v>
@@ -1407,7 +1407,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R19" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S19" t="str">
         <v>cmr9eluns000ha0igjf3iqgew</v>
@@ -1460,7 +1460,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R20" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S20" t="str">
         <v>cmr9eluns000ia0igwz0qd2xx</v>
@@ -1513,7 +1513,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R21" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S21" t="str">
         <v>cmr9eluns000ja0igwzx8kfom</v>
@@ -1566,7 +1566,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R22" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S22" t="str">
         <v>cmr9eluns000ka0igmjncpixp</v>
@@ -1619,7 +1619,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R23" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S23" t="str">
         <v>cmr9eluns000la0igi244fubl</v>
@@ -1672,7 +1672,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R24" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S24" t="str">
         <v>cmr9eluns000ma0ig6a2ti67m</v>
@@ -1725,7 +1725,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R25" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S25" t="str">
         <v>cmr9eluns000na0igffn6mjm7</v>
@@ -1778,7 +1778,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R26" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S26" t="str">
         <v>cmr9eluns000oa0igph8dcmvd</v>
@@ -1831,7 +1831,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R27" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S27" t="str">
         <v>cmr9eluns000pa0igf50ulrut</v>
@@ -1884,7 +1884,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R28" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S28" t="str">
         <v>cmr9eluns000qa0ig5yk3ngxr</v>
@@ -1937,7 +1937,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R29" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S29" t="str">
         <v>cmr9eluns000ra0ig2t8dsolc</v>
@@ -1990,7 +1990,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R30" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S30" t="str">
         <v>cmr9eluns000sa0ig2ten27rn</v>
@@ -2043,7 +2043,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R31" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S31" t="str">
         <v>cmr9eluns000ta0igbqzteqg8</v>
@@ -2096,7 +2096,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R32" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S32" t="str">
         <v>cmr9eluns000ua0iguw3egv1b</v>
@@ -2149,7 +2149,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R33" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S33" t="str">
         <v>cmr9eluns000va0igy9c1ucza</v>
@@ -2202,7 +2202,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R34" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S34" t="str">
         <v>cmr9eluns000wa0igasufikjt</v>
@@ -2255,7 +2255,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R35" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S35" t="str">
         <v>cmr9eluns000xa0ig86couhyr</v>
@@ -2308,7 +2308,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R36" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S36" t="str">
         <v>cmr9eluns000ya0ig5mj81cdj</v>
@@ -2361,7 +2361,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R37" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S37" t="str">
         <v>cmr9eluns000za0ig1n8p3gws</v>
@@ -2414,7 +2414,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R38" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S38" t="str">
         <v>cmr9elunt0010a0igawtolobu</v>
@@ -2467,7 +2467,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R39" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S39" t="str">
         <v>cmr9elunt0011a0igemqg52kg</v>
@@ -2520,7 +2520,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R40" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S40" t="str">
         <v>cmr9elunt0012a0igkrikbpeo</v>
@@ -2576,7 +2576,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R41" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S41" t="str">
         <v>cmr9elunt0013a0ig04gij873</v>
@@ -2629,7 +2629,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R42" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S42" t="str">
         <v>cmr9elunt0014a0igxkjt4ajy</v>
@@ -2682,7 +2682,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R43" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S43" t="str">
         <v>cmr9elunt0015a0igjsuvhvzz</v>
@@ -2735,7 +2735,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R44" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S44" t="str">
         <v>cmr9elunt0016a0igla5kplem</v>
@@ -2788,7 +2788,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R45" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S45" t="str">
         <v>cmr9elunt0017a0igzh9z2rpn</v>
@@ -2841,7 +2841,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R46" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S46" t="str">
         <v>cmr9elunt0018a0ig3u4ti3qi</v>
@@ -2894,7 +2894,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R47" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S47" t="str">
         <v>cmr9elunt0019a0ig1r9zj7cj</v>
@@ -2947,7 +2947,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R48" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S48" t="str">
         <v>cmr9elunt001aa0igltpr5ek9</v>
@@ -3000,7 +3000,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R49" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S49" t="str">
         <v>cmr9elunt001ba0igag1dllob</v>
@@ -3053,7 +3053,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R50" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S50" t="str">
         <v>cmr9elunt001ca0igs8wtzqws</v>
@@ -3106,7 +3106,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R51" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S51" t="str">
         <v>cmr9elunt001da0igst8asyxo</v>
@@ -3159,7 +3159,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R52" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S52" t="str">
         <v>cmr9elunt001ea0igozqz7l26</v>
@@ -3212,7 +3212,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R53" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S53" t="str">
         <v>cmr9elunt001fa0ig02bxd98v</v>
@@ -3265,7 +3265,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R54" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S54" t="str">
         <v>cmr9elunt001ga0igbnere9pk</v>
@@ -3318,7 +3318,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R55" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S55" t="str">
         <v>cmr9elunt001ha0igjeu5mu08</v>
@@ -3371,7 +3371,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R56" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S56" t="str">
         <v>cmr9elunt001ia0igyetq1gpj</v>
@@ -3424,7 +3424,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R57" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S57" t="str">
         <v>cmr9elunt001ja0igovjhrqtn</v>
@@ -3477,7 +3477,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R58" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S58" t="str">
         <v>cmr9elunt001ka0ig75z3u6c5</v>
@@ -3530,7 +3530,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R59" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S59" t="str">
         <v>cmr9elunt001la0igcbht2rx4</v>
@@ -3583,7 +3583,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R60" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S60" t="str">
         <v>cmr9elunt001ma0igain7iv0v</v>
@@ -3636,7 +3636,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R61" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S61" t="str">
         <v>cmr9elunu001na0igvhxq19l4</v>
@@ -3689,7 +3689,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R62" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S62" t="str">
         <v>cmr9elunu001oa0igqct1mt94</v>
@@ -3742,7 +3742,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R63" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S63" t="str">
         <v>cmr9elunu001pa0igpfo3c8th</v>
@@ -3795,7 +3795,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R64" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S64" t="str">
         <v>cmr9elunu001qa0igvdba97nz</v>
@@ -3848,7 +3848,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R65" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S65" t="str">
         <v>cmr9elunu001ra0igogdyrhbb</v>
@@ -3901,7 +3901,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R66" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S66" t="str">
         <v>cmr9elunu001sa0igbv6dcn38</v>
@@ -3954,7 +3954,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R67" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S67" t="str">
         <v>cmr9elunu001ta0igg3v3lk78</v>
@@ -4007,7 +4007,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R68" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S68" t="str">
         <v>cmr9elunu001ua0ig9wo5h8ka</v>
@@ -4060,7 +4060,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R69" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S69" t="str">
         <v>cmr9elunu001va0igbsrfqjw0</v>
@@ -4113,7 +4113,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R70" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S70" t="str">
         <v>cmr9elunu001wa0igfemdmfpq</v>
@@ -4166,7 +4166,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R71" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S71" t="str">
         <v>cmr9elunu001xa0ign17p5dx2</v>
@@ -4219,7 +4219,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R72" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S72" t="str">
         <v>cmr9elunu001ya0iglm2doypy</v>
@@ -4272,7 +4272,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R73" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S73" t="str">
         <v>cmr9elunu001za0ighgyrb6fy</v>
@@ -4325,7 +4325,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R74" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S74" t="str">
         <v>cmr9elunu0020a0igm50jolui</v>
@@ -4378,7 +4378,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R75" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S75" t="str">
         <v>cmr9elunu0021a0igvbw1uziz</v>
@@ -4431,7 +4431,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R76" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S76" t="str">
         <v>cmr9elunu0022a0igofbtsxqn</v>
@@ -4484,7 +4484,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R77" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S77" t="str">
         <v>cmr9elunu0023a0igup8ejach</v>
@@ -4537,7 +4537,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R78" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S78" t="str">
         <v>cmr9elunu0024a0igvuj78wti</v>
@@ -4590,7 +4590,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R79" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S79" t="str">
         <v>cmr9elunu0025a0igw3cxru8f</v>
@@ -4643,7 +4643,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R80" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S80" t="str">
         <v>cmr9elunu0026a0ignq7ntxih</v>
@@ -4696,7 +4696,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R81" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S81" t="str">
         <v>cmr9elunu0027a0igf293zj4w</v>
@@ -4749,7 +4749,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R82" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S82" t="str">
         <v>cmr9elunu0028a0igu5m3lxlh</v>
@@ -4802,7 +4802,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R83" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S83" t="str">
         <v>cmr9elunu0029a0ig701g2hby</v>
@@ -4855,7 +4855,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R84" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S84" t="str">
         <v>cmr9elunu002aa0igxnstqxcg</v>
@@ -4908,7 +4908,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R85" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S85" t="str">
         <v>cmr9elunu002ba0ign8nfsrqm</v>
@@ -4961,7 +4961,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R86" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S86" t="str">
         <v>cmr9elunu002ca0iglyzuncts</v>
@@ -5014,7 +5014,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R87" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S87" t="str">
         <v>cmr9elunu002da0iggm3ajcdb</v>
@@ -5067,7 +5067,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R88" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S88" t="str">
         <v>cmr9elunu002ea0igxxdkeg4j</v>
@@ -5120,7 +5120,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R89" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S89" t="str">
         <v>cmr9elunu002fa0ig3gk0au6g</v>
@@ -5173,7 +5173,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R90" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S90" t="str">
         <v>cmr9elunu002ga0ig4grxx3cp</v>
@@ -5226,7 +5226,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R91" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S91" t="str">
         <v>cmr9elunu002ha0igoje31em3</v>
@@ -5279,7 +5279,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R92" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S92" t="str">
         <v>cmr9elunu002ia0ig4dalffqr</v>
@@ -5332,7 +5332,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R93" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S93" t="str">
         <v>cmr9elunu002ja0ig6x6ovjid</v>
@@ -5385,7 +5385,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R94" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S94" t="str">
         <v>cmr9elunu002ka0ig9kyxa0q5</v>
@@ -5438,7 +5438,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R95" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S95" t="str">
         <v>cmr9elunu002la0igcvxmflks</v>
@@ -5491,7 +5491,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R96" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S96" t="str">
         <v>cmr9elunu002ma0ig2htx7br6</v>
@@ -5544,7 +5544,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R97" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S97" t="str">
         <v>cmr9elunu002na0igwtyw1inx</v>
@@ -5597,7 +5597,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R98" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S98" t="str">
         <v>cmr9elunu002oa0ig59s4ouzx</v>
@@ -5650,7 +5650,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R99" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S99" t="str">
         <v>cmr9elunu002pa0igtn21fsfs</v>
@@ -5703,7 +5703,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R100" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S100" t="str">
         <v>cmr9elunu002qa0igmv5shs30</v>
@@ -5756,7 +5756,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R101" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S101" t="str">
         <v>cmr9elunu002ra0igavsslwon</v>
@@ -5809,7 +5809,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R102" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S102" t="str">
         <v>cmr9elunu002sa0igh5y6yn2g</v>
@@ -5862,7 +5862,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R103" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S103" t="str">
         <v>cmr9elunu002ta0ig3vanfcj2</v>
@@ -5915,7 +5915,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R104" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S104" t="str">
         <v>cmr9elunu002ua0ighpcc8mq0</v>
@@ -5968,7 +5968,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R105" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S105" t="str">
         <v>cmr9elunu002va0igsyih5jaz</v>
@@ -6021,7 +6021,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R106" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S106" t="str">
         <v>cmr9elunu002wa0igaxsums3a</v>
@@ -6074,7 +6074,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R107" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S107" t="str">
         <v>cmr9elunu002xa0ig6w5n18nh</v>
@@ -6127,7 +6127,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R108" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S108" t="str">
         <v>cmr9elunu002ya0igptc7motz</v>
@@ -6180,7 +6180,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R109" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S109" t="str">
         <v>cmr9elunu002za0iguyuqqi7k</v>
@@ -6233,7 +6233,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R110" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S110" t="str">
         <v>cmr9elunu0030a0ig4e5zrngj</v>
@@ -6286,7 +6286,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R111" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S111" t="str">
         <v>cmr9elunu0031a0ig1kbwcrkq</v>
@@ -6339,7 +6339,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R112" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S112" t="str">
         <v>cmr9elunv0032a0igqr2ug2p5</v>
@@ -6392,7 +6392,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R113" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S113" t="str">
         <v>cmr9elunv0033a0igp0fbtx1i</v>
@@ -6445,7 +6445,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R114" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S114" t="str">
         <v>cmr9elunv0034a0igtajr11er</v>
@@ -6498,7 +6498,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R115" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S115" t="str">
         <v>cmr9elunv0035a0igi8k6s9q2</v>
@@ -6551,7 +6551,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R116" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S116" t="str">
         <v>cmr9elunv0036a0igkzud6dos</v>
@@ -6604,7 +6604,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R117" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S117" t="str">
         <v>cmr9elunv0037a0ignj02gpb6</v>
@@ -6657,7 +6657,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R118" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S118" t="str">
         <v>cmr9elunv0038a0ig9ahyplfp</v>
@@ -6710,7 +6710,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R119" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S119" t="str">
         <v>cmr9elunv0039a0igbcil7o8i</v>
@@ -6763,7 +6763,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R120" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S120" t="str">
         <v>cmr9elunv003aa0igkd2ewg93</v>
@@ -6816,7 +6816,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R121" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S121" t="str">
         <v>cmr9elunv003ba0ig1ewm1c10</v>
@@ -6869,7 +6869,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R122" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S122" t="str">
         <v>cmr9elunv003ca0igx1gou9pu</v>
@@ -6922,7 +6922,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R123" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S123" t="str">
         <v>cmr9elunv003da0iggji1541t</v>
@@ -6975,7 +6975,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R124" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S124" t="str">
         <v>cmr9elunv003ea0igkp35kfmq</v>
@@ -7028,7 +7028,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R125" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S125" t="str">
         <v>cmr9elunv003fa0igk4ed5dsq</v>
@@ -7081,7 +7081,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R126" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S126" t="str">
         <v>cmr9elunv003ga0ig3tero7y5</v>
@@ -7134,7 +7134,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R127" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S127" t="str">
         <v>cmr9elunv003ha0igswrskv23</v>
@@ -7187,7 +7187,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R128" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S128" t="str">
         <v>cmr9elunv003ia0ighlz7hahn</v>
@@ -7240,7 +7240,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R129" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S129" t="str">
         <v>cmr9elunv003ja0ig077lzwqk</v>
@@ -7293,7 +7293,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R130" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S130" t="str">
         <v>cmr9elunv003ka0iguvcbzox1</v>
@@ -7346,7 +7346,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R131" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S131" t="str">
         <v>cmr9elunv003la0igora3a9v7</v>
@@ -7399,7 +7399,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R132" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S132" t="str">
         <v>cmr9elunv003ma0ig6zdxuz6q</v>
@@ -7452,7 +7452,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R133" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S133" t="str">
         <v>cmr9elunv003na0igzl9ulayp</v>
@@ -7505,7 +7505,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R134" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S134" t="str">
         <v>cmr9elunv003oa0igw1mqsy59</v>
@@ -7558,7 +7558,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R135" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S135" t="str">
         <v>cmr9elunv003pa0ig093i3m7p</v>
@@ -7611,7 +7611,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R136" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S136" t="str">
         <v>cmr9elunv003qa0ig3lfxfs15</v>
@@ -7664,7 +7664,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R137" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S137" t="str">
         <v>cmr9elunv003ra0iguzimlgid</v>
@@ -7717,7 +7717,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R138" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S138" t="str">
         <v>cmr9elunv003sa0igvjdle4sl</v>
@@ -7770,7 +7770,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R139" s="1">
-        <v>46209.45660759259</v>
+        <v>46209.66507981481</v>
       </c>
       <c r="S139" t="str">
         <v>cmr9elunv003ta0igeabm1qsu</v>
@@ -7823,7 +7823,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R140" s="1">
-        <v>46261.462280486114</v>
+        <v>46261.670752708334</v>
       </c>
       <c r="S140" t="str">
         <v>cmtbpsnii000004li6br5az93</v>
@@ -7876,7 +7876,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R141" s="1">
-        <v>46261.46357652778</v>
+        <v>46261.67204875</v>
       </c>
       <c r="S141" t="str">
         <v>cmtbpv1wz000304li9k9yskwt</v>
@@ -7932,7 +7932,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R142" s="1">
-        <v>46261.46633523148</v>
+        <v>46261.6748074537</v>
       </c>
       <c r="S142" t="str">
         <v>cmtbq05tv000004l85hzj4y38</v>
@@ -7988,7 +7988,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R143" s="1">
-        <v>46254.51726792824</v>
+        <v>46254.72574015046</v>
       </c>
       <c r="S143" t="str">
         <v>cmt1sjiod000604jzt4ksugtf</v>
@@ -8044,7 +8044,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R144" s="1">
-        <v>46261.46657258102</v>
+        <v>46261.67504480324</v>
       </c>
       <c r="S144" t="str">
         <v>cmtbq0lnj000304l8drjdaw8i</v>
@@ -8097,7 +8097,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R145" s="1">
-        <v>46261.4675221875</v>
+        <v>46261.67599440972</v>
       </c>
       <c r="S145" t="str">
         <v>cmtbq2cyl000904lik4fddeeb</v>
@@ -8150,7 +8150,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R146" s="1">
-        <v>46261.467995844905</v>
+        <v>46261.67646806713</v>
       </c>
       <c r="S146" t="str">
         <v>cmtbq38jd000c04lig4h0cc0j</v>
@@ -8203,7 +8203,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R147" s="1">
-        <v>46261.468583368056</v>
+        <v>46261.67705559028</v>
       </c>
       <c r="S147" t="str">
         <v>cmtbq4bpf000f04litdssdkfc</v>
@@ -8256,7 +8256,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R148" s="1">
-        <v>46261.46903818287</v>
+        <v>46261.67751040509</v>
       </c>
       <c r="S148" t="str">
         <v>cmtbq560z000j04ligruly4np</v>
@@ -8309,7 +8309,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R149" s="1">
-        <v>46261.46644855324</v>
+        <v>46261.67492077546</v>
       </c>
       <c r="S149" t="str">
         <v>cmtbq0ddv000604lizkwpbocj</v>
@@ -8362,7 +8362,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R150" s="1">
-        <v>46261.46929712963</v>
+        <v>46261.67776935185</v>
       </c>
       <c r="S150" t="str">
         <v>cmtbq5nag000604l8cahh5kco</v>
@@ -8415,7 +8415,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R151" s="1">
-        <v>46238.616294085645</v>
+        <v>46238.82476630787</v>
       </c>
       <c r="S151" t="str">
         <v>cmsf2l9r5000104jwko4a6i8i</v>
@@ -8471,7 +8471,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R152" s="1">
-        <v>46223.629137777774</v>
+        <v>46223.83761</v>
       </c>
       <c r="S152" t="str">
         <v>cmrtnna00000004jsmn9e3b8h</v>
@@ -8524,7 +8524,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R153" s="1">
-        <v>46223.62931563657</v>
+        <v>46223.8377878588</v>
       </c>
       <c r="S153" t="str">
         <v>cmrtnnluv000004jy0vs5h1kr</v>
@@ -8580,7 +8580,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R154" s="1">
-        <v>46223.62946474537</v>
+        <v>46223.83793696759</v>
       </c>
       <c r="S154" t="str">
         <v>cmrtnnvsq000304jymet30t9b</v>
@@ -8636,7 +8636,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R155" s="1">
-        <v>46254.51595956019</v>
+        <v>46254.72443178241</v>
       </c>
       <c r="S155" t="str">
         <v>cmt1sh3ga000004l1jmbap7g3</v>
@@ -8692,7 +8692,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R156" s="1">
-        <v>46254.560680393515</v>
+        <v>46254.76915261574</v>
       </c>
       <c r="S156" t="str">
         <v>cmt1urwua000204l7jj43mppg</v>
@@ -8745,7 +8745,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R157" s="1">
-        <v>46254.52901197917</v>
+        <v>46254.73748420139</v>
       </c>
       <c r="S157" t="str">
         <v>cmt1t59m3000004joo687y3fa</v>
@@ -8798,7 +8798,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R158" s="1">
-        <v>46254.51701357639</v>
+        <v>46254.72548579861</v>
       </c>
       <c r="S158" t="str">
         <v>cmt1sj1px000304jzoeruz4c9</v>
@@ -8851,7 +8851,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R159" s="1">
-        <v>46223.63124967593</v>
+        <v>46223.83972189815</v>
       </c>
       <c r="S159" t="str">
         <v>cmrtnr6sk000904jyw49ijwbm</v>
@@ -8907,7 +8907,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R160" s="1">
-        <v>46238.57922263889</v>
+        <v>46238.78769486111</v>
       </c>
       <c r="S160" t="str">
         <v>cmsf0ombo000c04i5yu5pnwc7</v>
@@ -8960,7 +8960,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R161" s="1">
-        <v>46238.579439814814</v>
+        <v>46238.787912037034</v>
       </c>
       <c r="S161" t="str">
         <v>cmsf0p0sv000004l8gfzfw0jy</v>
@@ -9013,7 +9013,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R162" s="1">
-        <v>46238.57968923611</v>
+        <v>46238.78816145833</v>
       </c>
       <c r="S162" t="str">
         <v>cmsf0phfi000f04i52ftu4kda</v>
@@ -9069,7 +9069,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R163" s="1">
-        <v>46238.57895025463</v>
+        <v>46238.78742247685</v>
       </c>
       <c r="S163" t="str">
         <v>cmsf0o45y000904i5vs7efhqq</v>
@@ -9122,7 +9122,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R164" s="1">
-        <v>46239.3856490625</v>
+        <v>46239.594121284725</v>
       </c>
       <c r="S164" t="str">
         <v>cmsg66033000304l771xe9zie</v>
@@ -9175,7 +9175,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R165" s="1">
-        <v>46223.64234229166</v>
+        <v>46223.85081451389</v>
       </c>
       <c r="S165" t="str">
         <v>cmrtobqau000304jyoq3lqt8d</v>
@@ -9228,7 +9228,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R166" s="1">
-        <v>46223.62113543982</v>
+        <v>46223.82960766204</v>
       </c>
       <c r="S166" t="str">
         <v>cmrtn8gid000004l1i87h6r0n</v>
@@ -9284,7 +9284,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R167" s="1">
-        <v>46238.6682516088</v>
+        <v>46238.87672383102</v>
       </c>
       <c r="S167" t="str">
         <v>cmsf59hl7000004lbb0w3ra8n</v>
@@ -9340,7 +9340,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R168" s="1">
-        <v>46254.51628800926</v>
+        <v>46254.72476023148</v>
       </c>
       <c r="S168" t="str">
         <v>cmt1shpck000304l1n0zimm8u</v>
@@ -9393,7 +9393,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R169" s="1">
-        <v>46223.62993481482</v>
+        <v>46223.83840703704</v>
       </c>
       <c r="S169" t="str">
         <v>cmrtnor4w000604jy45p8ium3</v>
@@ -9446,7 +9446,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R170" s="1">
-        <v>46223.62125802083</v>
+        <v>46223.82973024306</v>
       </c>
       <c r="S170" t="str">
         <v>cmrtn8ool000304l1khbxdtpb</v>
@@ -9499,7 +9499,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R171" s="1">
-        <v>46238.57470483796</v>
+        <v>46238.783177060184</v>
       </c>
       <c r="S171" t="str">
         <v>cmsf0g94y000304i5wo0o70z9</v>
@@ -9555,7 +9555,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R172" s="1">
-        <v>46238.575018414354</v>
+        <v>46238.783490636575</v>
       </c>
       <c r="S172" t="str">
         <v>cmsf0gu1j000004jun1dxonqy</v>
@@ -9611,7 +9611,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R173" s="1">
-        <v>46254.515226793985</v>
+        <v>46254.723699016206</v>
       </c>
       <c r="S173" t="str">
         <v>cmt1sfqln000004jzjdprbwxo</v>
@@ -9667,7 +9667,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R174" s="1">
-        <v>46238.574272847225</v>
+        <v>46238.782745069446</v>
       </c>
       <c r="S174" t="str">
         <v>cmsf0fgc6000004i5owk7auie</v>
@@ -9723,7 +9723,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R175" s="1">
-        <v>46238.57858356481</v>
+        <v>46238.787055787034</v>
       </c>
       <c r="S175" t="str">
         <v>cmsf0nfpw000604i5y82b9zvh</v>
@@ -9776,7 +9776,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R176" s="1">
-        <v>46223.604721979165</v>
+        <v>46223.813194201386</v>
       </c>
       <c r="S176" t="str">
         <v>cmrtme2a3000004jxv5gf96lh</v>
@@ -9829,7 +9829,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R177" s="1">
-        <v>46223.60494292824</v>
+        <v>46223.813415150464</v>
       </c>
       <c r="S177" t="str">
         <v>cmrtmeh0c000004jmhl08l1yr</v>
@@ -9882,7 +9882,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R178" s="1">
-        <v>46223.605333541665</v>
+        <v>46223.813805763886</v>
       </c>
       <c r="S178" t="str">
         <v>cmrtmf71u000304jm1m2dtqbd</v>
@@ -9935,7 +9935,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R179" s="1">
-        <v>46223.606342997686</v>
+        <v>46223.81481521991</v>
       </c>
       <c r="S179" t="str">
         <v>cmrtmh2cj000304jx8z1h4ona</v>
@@ -9988,7 +9988,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R180" s="1">
-        <v>46223.64178064815</v>
+        <v>46223.85025287037</v>
       </c>
       <c r="S180" t="str">
         <v>cmrtoaouw000004jytaq7sxyl</v>
@@ -10044,7 +10044,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R181" s="1">
-        <v>46223.55316135417</v>
+        <v>46223.76163357639</v>
       </c>
       <c r="S181" t="str">
         <v>cmrtjqkwl000704jxy2n161s5</v>
@@ -10100,7 +10100,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R182" s="1">
-        <v>46223.55340459491</v>
+        <v>46223.76187681713</v>
       </c>
       <c r="S182" t="str">
         <v>cmrtjr14d000a04jxnm0cmwlr</v>
@@ -10153,7 +10153,7 @@
         <v>user-sesacre</v>
       </c>
       <c r="R183" s="1">
-        <v>46223.564256909725</v>
+        <v>46223.772729131946</v>
       </c>
       <c r="S183" t="str">
         <v>cmrtkb4lx000004kztfr1m1ej</v>
@@ -10209,7 +10209,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R184" s="1">
-        <v>46223.55547172454</v>
+        <v>46223.76394394676</v>
       </c>
       <c r="S184" t="str">
         <v>cmrtjuuxh000d04jxkeypwsw3</v>
@@ -10265,7 +10265,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R185" s="1">
-        <v>46223.555669375</v>
+        <v>46223.764141597225</v>
       </c>
       <c r="S185" t="str">
         <v>cmrtjv83u000g04jxphnd9fqb</v>
@@ -10318,7 +10318,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R186" s="1">
-        <v>46265.53331241898</v>
+        <v>46265.741784641206</v>
       </c>
       <c r="S186" t="str">
         <v>cmthj7ln5000004lcsye9k1h2</v>
@@ -10371,7 +10371,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R187" s="1">
-        <v>46265.53346414352</v>
+        <v>46265.74193636574</v>
       </c>
       <c r="S187" t="str">
         <v>cmthj7vra000304lcs18i2dtk</v>
@@ -10427,7 +10427,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R188" s="1">
-        <v>46265.53377681713</v>
+        <v>46265.74224903935</v>
       </c>
       <c r="S188" t="str">
         <v>cmthj8glp000904lccyavujjg</v>
@@ -10483,7 +10483,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R189" s="1">
-        <v>46239.39483556713</v>
+        <v>46239.60330778935</v>
       </c>
       <c r="S189" t="str">
         <v>cmsg6n0ip000004jr7ds29exx</v>
@@ -10539,7 +10539,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R190" s="1">
-        <v>46265.53365486111</v>
+        <v>46265.74212708334</v>
       </c>
       <c r="S190" t="str">
         <v>cmthj88h0000604lcylq634f9</v>
@@ -10595,7 +10595,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R191" s="1">
-        <v>46265.53311974537</v>
+        <v>46265.74159196759</v>
       </c>
       <c r="S191" t="str">
         <v>cmthj78sq000104l3gfmp0jgc</v>
@@ -10648,7 +10648,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R192" s="1">
-        <v>46265.531889224534</v>
+        <v>46265.74036144676</v>
       </c>
       <c r="S192" t="str">
         <v>cmthj4yrh000004l8a69veuyo</v>
@@ -10701,7 +10701,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R193" s="1">
-        <v>46265.535834814815</v>
+        <v>46265.744307037035</v>
       </c>
       <c r="S193" t="str">
         <v>cmthjc9sw000604lf4cn4vwt5</v>
@@ -10754,7 +10754,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R194" s="1">
-        <v>46265.53606391203</v>
+        <v>46265.74453613426</v>
       </c>
       <c r="S194" t="str">
         <v>cmthjcp2q000904lfarq7elp3</v>
@@ -10810,7 +10810,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R195" s="1">
-        <v>46238.605248182874</v>
+        <v>46238.813720405095</v>
       </c>
       <c r="S195" t="str">
         <v>cmsf20tcz000604l6x1xwlflq</v>
@@ -10866,7 +10866,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R196" s="1">
-        <v>46238.60538221065</v>
+        <v>46238.81385443287</v>
       </c>
       <c r="S196" t="str">
         <v>cmsf212an000304jyvevuox9q</v>
@@ -10922,7 +10922,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R197" s="1">
-        <v>46238.60560940972</v>
+        <v>46238.81408163194</v>
       </c>
       <c r="S197" t="str">
         <v>cmsf21hfx000904l6buvlz5ru</v>
@@ -10975,7 +10975,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R198" s="1">
-        <v>46238.59723115741</v>
+        <v>46238.80570337963</v>
       </c>
       <c r="S198" t="str">
         <v>cmsf1lyw4000004l6por9dm1h</v>
@@ -11031,7 +11031,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R199" s="1">
-        <v>46238.601645925926</v>
+        <v>46238.81011814815</v>
       </c>
       <c r="S199" t="str">
         <v>cmsf1u57k000204jr07okwft0</v>
@@ -11087,7 +11087,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R200" s="1">
-        <v>46238.60194810185</v>
+        <v>46238.81042032407</v>
       </c>
       <c r="S200" t="str">
         <v>cmsf1upcr000004jyekn2pm8q</v>
@@ -11143,7 +11143,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R201" s="1">
-        <v>46238.60211811343</v>
+        <v>46238.81059033565</v>
       </c>
       <c r="S201" t="str">
         <v>cmsf1v0ot000304l6hx1gnxev</v>
@@ -11199,7 +11199,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R202" s="1">
-        <v>46238.61266734954</v>
+        <v>46238.82113957176</v>
       </c>
       <c r="S202" t="str">
         <v>cmsf2ejyz000304l16vsyf12y</v>
@@ -11255,7 +11255,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R203" s="1">
-        <v>46238.605819212964</v>
+        <v>46238.814291435185</v>
       </c>
       <c r="S203" t="str">
         <v>cmsf21vfg000c04l67m17ulij</v>
@@ -11311,7 +11311,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R204" s="1">
-        <v>46238.60639381944</v>
+        <v>46238.81486604167</v>
       </c>
       <c r="S204" t="str">
         <v>cmsf22xqi000604jykcqqcmvx</v>
@@ -11367,7 +11367,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R205" s="1">
-        <v>46238.61213123843</v>
+        <v>46238.82060346065</v>
       </c>
       <c r="S205" t="str">
         <v>cmsf2dk8b000004l1nkn5uefj</v>
@@ -11423,7 +11423,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R206" s="1">
-        <v>46238.61250349537</v>
+        <v>46238.820975717594</v>
       </c>
       <c r="S206" t="str">
         <v>cmsf2e91q000904jyg5yyydie</v>
@@ -11476,7 +11476,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R207" s="1">
-        <v>46247.34303138889</v>
+        <v>46247.55150361111</v>
       </c>
       <c r="S207" t="str">
         <v>cmsrjhw8o000904jrjyha7iu9</v>
@@ -11529,7 +11529,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R208" s="1">
-        <v>46247.34400041667</v>
+        <v>46247.55247263889</v>
       </c>
       <c r="S208" t="str">
         <v>cmsrjjouc000c04jrawjz98v1</v>
@@ -11585,7 +11585,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R209" s="1">
-        <v>46247.34026386574</v>
+        <v>46247.54873608796</v>
       </c>
       <c r="S209" t="str">
         <v>cmsrjcrqm000004jr8uf1bvps</v>
@@ -11641,7 +11641,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R210" s="1">
-        <v>46247.34054914352</v>
+        <v>46247.54902136574</v>
       </c>
       <c r="S210" t="str">
         <v>cmsrjdara000304jrlze4ix9x</v>
@@ -11697,7 +11697,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R211" s="1">
-        <v>46247.33984357639</v>
+        <v>46247.54831579861</v>
       </c>
       <c r="S211" t="str">
         <v>cmsrjbzpx000004ju48z6e1ja</v>
@@ -11753,7 +11753,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R212" s="1">
-        <v>46247.34116832176</v>
+        <v>46247.549640543984</v>
       </c>
       <c r="S212" t="str">
         <v>cmsrjeg1b000604jrels0je5u</v>
@@ -11809,7 +11809,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R213" s="1">
-        <v>46238.62990986111</v>
+        <v>46238.83838208333</v>
       </c>
       <c r="S213" t="str">
         <v>cmsf3ahh0000004jo3gg0irst</v>
@@ -11865,7 +11865,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R214" s="1">
-        <v>46238.63009381945</v>
+        <v>46238.83856604167</v>
       </c>
       <c r="S214" t="str">
         <v>cmsf3atqi000004l3m7awoz6w</v>
@@ -11921,7 +11921,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R215" s="1">
-        <v>46238.63020224537</v>
+        <v>46238.838674467595</v>
       </c>
       <c r="S215" t="str">
         <v>cmsf3b0yq000304l3802xhkvf</v>
@@ -11977,7 +11977,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R216" s="1">
-        <v>46238.6305815625</v>
+        <v>46238.83905378472</v>
       </c>
       <c r="S216" t="str">
         <v>cmsf3bq93000604l3ajez33hc</v>
@@ -12033,7 +12033,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R217" s="1">
-        <v>46238.63094375</v>
+        <v>46238.83941597222</v>
       </c>
       <c r="S217" t="str">
         <v>cmsf3ceec000904l3p6b7yl0r</v>
@@ -12089,7 +12089,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R218" s="1">
-        <v>46238.631456076386</v>
+        <v>46238.839928298614</v>
       </c>
       <c r="S218" t="str">
         <v>cmsf3dcjx000c04l3cjsjd0ex</v>
@@ -12145,7 +12145,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R219" s="1">
-        <v>46238.6323500463</v>
+        <v>46238.84082226852</v>
       </c>
       <c r="S219" t="str">
         <v>cmsf3f05g000304jomxbza6i7</v>
@@ -12201,7 +12201,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R220" s="1">
-        <v>46238.63249856482</v>
+        <v>46238.84097078704</v>
       </c>
       <c r="S220" t="str">
         <v>cmsf3fa1w000604jo827vhgjg</v>
@@ -12257,7 +12257,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R221" s="1">
-        <v>46238.63787305556</v>
+        <v>46238.84634527778</v>
       </c>
       <c r="S221" t="str">
         <v>cmsf3p8co000004l478i0am7j</v>
@@ -12313,7 +12313,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R222" s="1">
-        <v>46238.63806217592</v>
+        <v>46238.84653439815</v>
       </c>
       <c r="S222" t="str">
         <v>cmsf3pkyk000004jru7fj004g</v>
@@ -12369,7 +12369,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R223" s="1">
-        <v>46238.638240416665</v>
+        <v>46238.846712638886</v>
       </c>
       <c r="S223" t="str">
         <v>cmsf3pwuc000304jro7nwqnjj</v>
@@ -12425,7 +12425,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R224" s="1">
-        <v>46238.63835803241</v>
+        <v>46238.84683025463</v>
       </c>
       <c r="S224" t="str">
         <v>cmsf3q4om000004i52bxff9nd</v>
@@ -12481,7 +12481,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R225" s="1">
-        <v>46238.638504456016</v>
+        <v>46238.846976678244</v>
       </c>
       <c r="S225" t="str">
         <v>cmsf3qeg1000304i5wwgfleu0</v>
@@ -12537,7 +12537,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R226" s="1">
-        <v>46238.638884479165</v>
+        <v>46238.847356701386</v>
       </c>
       <c r="S226" t="str">
         <v>cmsf3r3s3000604i5s5nrcfuk</v>
@@ -12593,7 +12593,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R227" s="1">
-        <v>46238.63920423611</v>
+        <v>46238.84767645833</v>
       </c>
       <c r="S227" t="str">
         <v>cmsf3rp3i000904i5y4jzhpwr</v>
@@ -12649,7 +12649,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R228" s="1">
-        <v>46238.63947625</v>
+        <v>46238.84794847222</v>
       </c>
       <c r="S228" t="str">
         <v>cmsf3s78c000c04i5ijwn2fk6</v>
@@ -12705,7 +12705,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R229" s="1">
-        <v>46238.639700844906</v>
+        <v>46238.84817306713</v>
       </c>
       <c r="S229" t="str">
         <v>cmsf3sm7d000604jrfe80xmqc</v>
@@ -12761,7 +12761,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R230" s="1">
-        <v>46238.63982849537</v>
+        <v>46238.84830071759</v>
       </c>
       <c r="S230" t="str">
         <v>cmsf3supq000904jrmnybw4s2</v>
@@ -12817,7 +12817,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R231" s="1">
-        <v>46239.396318784726</v>
+        <v>46239.60479100695</v>
       </c>
       <c r="S231" t="str">
         <v>cmsg6pref000004kzjrwqno1j</v>
@@ -12873,7 +12873,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R232" s="1">
-        <v>46238.640205208336</v>
+        <v>46238.84867743056</v>
       </c>
       <c r="S232" t="str">
         <v>cmsf3tjtu000c04jrwiw7ht8a</v>
@@ -12929,7 +12929,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R233" s="1">
-        <v>46238.64036135417</v>
+        <v>46238.84883357639</v>
       </c>
       <c r="S233" t="str">
         <v>cmsf3tu8l000f04jr31izk3aa</v>
@@ -12985,7 +12985,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R234" s="1">
-        <v>46238.64049980324</v>
+        <v>46238.848972025466</v>
       </c>
       <c r="S234" t="str">
         <v>cmsf3u3gv000i04jr48nmwsdl</v>
@@ -13041,7 +13041,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R235" s="1">
-        <v>46238.640770833335</v>
+        <v>46238.849243055556</v>
       </c>
       <c r="S235" t="str">
         <v>cmsf3uljc000f04i5zpyhh1ih</v>
@@ -13097,7 +13097,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R236" s="1">
-        <v>46238.640964108796</v>
+        <v>46238.84943633102</v>
       </c>
       <c r="S236" t="str">
         <v>cmsf3uyf7000i04i5f8ksst9w</v>
@@ -13153,7 +13153,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R237" s="1">
-        <v>46238.641185925924</v>
+        <v>46238.849658148145</v>
       </c>
       <c r="S237" t="str">
         <v>cmsf3vd7k000l04i54fbl2gcq</v>
@@ -13209,7 +13209,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R238" s="1">
-        <v>46251.582144513886</v>
+        <v>46251.790616736114</v>
       </c>
       <c r="S238" t="str">
         <v>cmsxlk3s6000004jxkcma3szo</v>
@@ -13265,7 +13265,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R239" s="1">
-        <v>46251.58280427083</v>
+        <v>46251.79127649306</v>
       </c>
       <c r="S239" t="str">
         <v>cmsxllbrl000304jxpu4r9fll</v>
@@ -13321,7 +13321,7 @@
         <v>cmpr2e02k0001g8igkaf1ukhg</v>
       </c>
       <c r="R240" s="1">
-        <v>46213.61443601852</v>
+        <v>46213.82290824074</v>
       </c>
       <c r="S240" t="str">
         <v>cmrfchj7s000004lacd0ou74c</v>
@@ -13377,7 +13377,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R241" s="1">
-        <v>46239.391583275465</v>
+        <v>46239.600055497685</v>
       </c>
       <c r="S241" t="str">
         <v>cmsg6gzp6000a04kxwhqudztd</v>
@@ -13433,7 +13433,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R242" s="1">
-        <v>46239.39168409722</v>
+        <v>46239.600156319444</v>
       </c>
       <c r="S242" t="str">
         <v>cmsg6h6f6000d04kx1h0p2n3z</v>
@@ -13489,7 +13489,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R243" s="1">
-        <v>46239.391798668985</v>
+        <v>46239.600270891206</v>
       </c>
       <c r="S243" t="str">
         <v>cmsg6he25000g04kx16nwjie0</v>
@@ -13545,7 +13545,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R244" s="1">
-        <v>46239.3919190625</v>
+        <v>46239.60039128472</v>
       </c>
       <c r="S244" t="str">
         <v>cmsg6hm33000004l50w5ygvqk</v>
@@ -13601,7 +13601,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R245" s="1">
-        <v>46239.39200923611</v>
+        <v>46239.600481458336</v>
       </c>
       <c r="S245" t="str">
         <v>cmsg6hs3i000304l5uczjehwq</v>
@@ -13657,7 +13657,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R246" s="1">
-        <v>46239.39213269676</v>
+        <v>46239.60060491898</v>
       </c>
       <c r="S246" t="str">
         <v>cmsg6i0bt000604l5xfig0jv9</v>
@@ -13713,7 +13713,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R247" s="1">
-        <v>46239.3922446875</v>
+        <v>46239.60071690972</v>
       </c>
       <c r="S247" t="str">
         <v>cmsg6i7sl000904l57z0fx8u0</v>
@@ -13769,7 +13769,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R248" s="1">
-        <v>46239.39239915509</v>
+        <v>46239.60087137731</v>
       </c>
       <c r="S248" t="str">
         <v>cmsg6ii3b000c04l5ezmbb6sz</v>
@@ -13825,7 +13825,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R249" s="1">
-        <v>46239.39250163194</v>
+        <v>46239.60097385417</v>
       </c>
       <c r="S249" t="str">
         <v>cmsg6iox9000j04kxxtxpb3q4</v>
@@ -13881,7 +13881,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R250" s="1">
-        <v>46239.39265190972</v>
+        <v>46239.60112413194</v>
       </c>
       <c r="S250" t="str">
         <v>cmsg6iyxx000f04l5jfjenqaq</v>
@@ -13937,7 +13937,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R251" s="1">
-        <v>46239.39275894676</v>
+        <v>46239.601231168985</v>
       </c>
       <c r="S251" t="str">
         <v>cmsg6j62t000i04l5jnrxek2q</v>
@@ -13993,7 +13993,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R252" s="1">
-        <v>46239.39288900463</v>
+        <v>46239.60136122685</v>
       </c>
       <c r="S252" t="str">
         <v>cmsg6jeqy000m04kxtw683yx4</v>
@@ -14049,7 +14049,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R253" s="1">
-        <v>46239.39295271991</v>
+        <v>46239.60142494213</v>
       </c>
       <c r="S253" t="str">
         <v>cmsg6jizv000l04l5ayxumg71</v>
@@ -14105,7 +14105,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R254" s="1">
-        <v>46239.393071238424</v>
+        <v>46239.601543460645</v>
       </c>
       <c r="S254" t="str">
         <v>cmsg6jqwb000p04kxbwdbpjd4</v>
@@ -14161,7 +14161,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R255" s="1">
-        <v>46239.39320017361</v>
+        <v>46239.60167239583</v>
       </c>
       <c r="S255" t="str">
         <v>cmsg6jzhr000s04kxrfga0b74</v>
@@ -14217,7 +14217,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R256" s="1">
-        <v>46239.39327042824</v>
+        <v>46239.60174265046</v>
       </c>
       <c r="S256" t="str">
         <v>cmsg6k46d000v04kxe154uz26</v>
@@ -14273,7 +14273,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R257" s="1">
-        <v>46239.39336231481</v>
+        <v>46239.60183453704</v>
       </c>
       <c r="S257" t="str">
         <v>cmsg6kaaw000y04kxmdwvogu2</v>
@@ -14329,7 +14329,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R258" s="1">
-        <v>46239.39344876158</v>
+        <v>46239.6019209838</v>
       </c>
       <c r="S258" t="str">
         <v>cmsg6kg2d001104kx3l3ocn86</v>
@@ -14385,7 +14385,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R259" s="1">
-        <v>46239.393530925925</v>
+        <v>46239.602003148146</v>
       </c>
       <c r="S259" t="str">
         <v>cmsg6kljk001404kxttqd96u4</v>
@@ -14441,7 +14441,7 @@
         <v>cmprd1s0l000004l57xdz4r5o</v>
       </c>
       <c r="R260" s="1">
-        <v>46239.393621689815</v>
+        <v>46239.602093912035</v>
       </c>
       <c r="S260" t="str">
         <v>cmsg6krle000o04l5qq1czrk6</v>

</xml_diff>